<commit_message>
GAUCHO05: align HS codes with previous GAUCHO declaration
Use TARIC codes and Czech wording from the previous GAUCHO clearance
for repeat items (ceramics 6912 00 25 10, chairs 9401 61 00 00,
take-away boxes 4819 50 00 00, parrilla 7323 93 00 90, etc.).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013kgPsLTRumkJ7okPbw8b4c
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_EL_GAUCHO_CZ_GAUCHO05.xlsx
+++ b/output/HS_Code_Summary_EL_GAUCHO_CZ_GAUCHO05.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:M47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -649,31 +649,31 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>3924 10 00</t>
+          <t>3924 10 00 19</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Big tray; Bread plate; Chimichurri cup; Peanut bowl; Caviar spoon</t>
+          <t>Bread plate; Chimichurri cup; Peanut bowl</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Velký plastový servírovací podnos; Melaminový talířek na chléb; Melaminová miska na chimichurri; Melaminová miska na arašídy; Lžička na kaviár</t>
+          <t>Talíř na chléb, kulatý černý, melamin; Miska na chimichurri, melamin; Miska na arašídy, melamin</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>20, 26, 48, 63, 64</t>
+          <t>26, 48, 63</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Melanine, Plastic</t>
+          <t>Melanine</t>
         </is>
       </c>
       <c r="G10" s="4" t="n">
-        <v>1836</v>
+        <v>1800</v>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
@@ -681,10 +681,10 @@
         </is>
       </c>
       <c r="I10" s="6" t="n">
-        <v>251.04</v>
+        <v>223</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>1738.8</v>
+        <v>1290</v>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
@@ -698,7 +698,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+          <t>Kód dle minulého proclení GAUCHO.</t>
         </is>
       </c>
     </row>
@@ -710,22 +710,22 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>3926 90 97</t>
+          <t>3924 10 00 90</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Pin</t>
+          <t>Big tray; Caviar spoon</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Plastový odznak</t>
+          <t>Velký plastový tác do restaurace; Lžička na kaviár, plast</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>20, 64</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="G11" s="4" t="n">
-        <v>150</v>
+        <v>36</v>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
@@ -742,10 +742,10 @@
         </is>
       </c>
       <c r="I11" s="6" t="n">
-        <v>0.63</v>
+        <v>28.04</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>120</v>
+        <v>448.8</v>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
@@ -759,7 +759,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+          <t>Kód dle minulého proclení GAUCHO. Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
         </is>
       </c>
     </row>
@@ -771,31 +771,31 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>4414 90 00</t>
+          <t>3926 90 97 90</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Picture frame S; Picture frame M; Picture frame L; Picture frame XL; Picture frame Oval</t>
+          <t>Pin</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Dřevěný rámeček na obrazy S; Dřevěný rámeček na obrazy M; Dřevěný rámeček na obrazy L; Dřevěný rámeček na obrazy XL; Dřevěný rámeček na obrazy oválný</t>
+          <t>Plastový odznak</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>39, 40, 41, 42, 43</t>
+          <t>51</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Wood</t>
+          <t>Plastic</t>
         </is>
       </c>
       <c r="G12" s="4" t="n">
-        <v>105</v>
+        <v>150</v>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
@@ -803,10 +803,10 @@
         </is>
       </c>
       <c r="I12" s="6" t="n">
-        <v>117</v>
+        <v>0.63</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>1375</v>
+        <v>120</v>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
@@ -818,7 +818,11 @@
           <t>Ne</t>
         </is>
       </c>
-      <c r="M12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>Kód dle minulého proclení GAUCHO. Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -828,22 +832,22 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>4419 90 00</t>
+          <t>4414 90 00</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Round wooden bread</t>
+          <t>Picture frame S; Picture frame M; Picture frame L; Picture frame XL; Picture frame Oval</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Kulaté dřevěné prkénko na chléb</t>
+          <t>Dřevěný rámeček na obrazy S; Dřevěný rámeček na obrazy M; Dřevěný rámeček na obrazy L; Dřevěný rámeček na obrazy XL; Dřevěný rámeček na obrazy oválný</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>39, 40, 41, 42, 43</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -852,7 +856,7 @@
         </is>
       </c>
       <c r="G13" s="4" t="n">
-        <v>200</v>
+        <v>105</v>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
@@ -860,10 +864,10 @@
         </is>
       </c>
       <c r="I13" s="6" t="n">
-        <v>170</v>
+        <v>117</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>760</v>
+        <v>1375</v>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
@@ -885,31 +889,31 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>4421 91 00</t>
+          <t>4419 20 90 00</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Toothpick</t>
+          <t>Round wooden bread</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Bambusová párátka (krabička)</t>
+          <t>Prkénko servírovací na chléb, kulaté, rubber wood</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>30</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Bamboo</t>
+          <t>Wood</t>
         </is>
       </c>
       <c r="G14" s="4" t="n">
-        <v>30</v>
+        <v>200</v>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
@@ -917,10 +921,10 @@
         </is>
       </c>
       <c r="I14" s="6" t="n">
-        <v>10</v>
+        <v>170</v>
       </c>
       <c r="J14" s="6" t="n">
-        <v>69</v>
+        <v>760</v>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
@@ -932,7 +936,11 @@
           <t>Ne</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr"/>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>Kód dle minulého proclení GAUCHO.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -942,31 +950,31 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>4819 10 00</t>
+          <t>4421 91 00 00</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Shot glass souvernir box</t>
+          <t>Toothpick</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Papírová dárková krabička na panáky</t>
+          <t>Bambusová párátka</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>32</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>Bamboo</t>
         </is>
       </c>
       <c r="G15" s="4" t="n">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
@@ -974,10 +982,10 @@
         </is>
       </c>
       <c r="I15" s="6" t="n">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>230</v>
+        <v>69</v>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
@@ -989,7 +997,11 @@
           <t>Ne</t>
         </is>
       </c>
-      <c r="M15" s="4" t="inlineStr"/>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>Kód dle minulého proclení GAUCHO.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -999,22 +1011,22 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>4819 20 00</t>
+          <t>4819 20 00 00</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Take away burger box; Take away steak box S; Take away steak box M; Take away steak box L; Steakknives souvenir box</t>
+          <t>Take away burger box; Take away steak box S; Take away steak box M; Take away steak box L; Shot glass souvernir box; Steakknives souvenir box</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Papírová krabička na burger; Papírová krabice na steak S (potištěná); Papírová krabice na steak M (potištěná); Papírová krabice na steak L (potištěná); Papírová dárková krabička na steakové nože</t>
+          <t>Skládací krabička na burgery; Skládací krabice na steak S, potištěná; Skládací krabice na steak M, potištěná; Skládací krabice na steak L, potištěná; Papírová dárková krabička na panáky; Papírová dárková krabička na steakové nože</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>6, 7, 8, 9, 15</t>
+          <t>6, 7, 8, 9, 14, 15</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -1023,7 +1035,7 @@
         </is>
       </c>
       <c r="G16" s="4" t="n">
-        <v>3002</v>
+        <v>3102</v>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
@@ -1031,10 +1043,10 @@
         </is>
       </c>
       <c r="I16" s="6" t="n">
-        <v>1230</v>
+        <v>1256</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>3994.6</v>
+        <v>4224.6</v>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
@@ -1113,22 +1125,22 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>4820 30 00</t>
+          <t>4819 50 00 00</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Bill Holder</t>
+          <t>Take away box 120m; Take away box 210m; Take away box 500m; Take away box 1070m</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Papírové desky na účet</t>
+          <t>Papírová krabička TAKE AWAY 120 ml s papírovým víčkem; Papírová krabička TAKE AWAY 210 ml s papírovým víčkem; Papírová krabička TAKE AWAY 500 ml s papírovým víčkem; Papírová krabička TAKE AWAY 1070 ml s papírovým víčkem</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>2, 3, 4, 5</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1137,7 +1149,7 @@
         </is>
       </c>
       <c r="G18" s="4" t="n">
-        <v>500</v>
+        <v>8100</v>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
@@ -1145,10 +1157,10 @@
         </is>
       </c>
       <c r="I18" s="6" t="n">
-        <v>22</v>
+        <v>172</v>
       </c>
       <c r="J18" s="6" t="n">
-        <v>100</v>
+        <v>1840</v>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
@@ -1160,7 +1172,11 @@
           <t>Ne</t>
         </is>
       </c>
-      <c r="M18" s="4" t="inlineStr"/>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>Kód dle minulého proclení GAUCHO.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1170,22 +1186,22 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>4823 69 90</t>
+          <t>4820 30 00</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Take away box 120m; Take away box 210m; Take away box 500m; Take away box 1070m</t>
+          <t>Bill Holder</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Papírová miska 120 ml s papírovým víčkem; Papírová miska 210 ml s papírovým víčkem; Papírová miska 500 ml s papírovým víčkem; Papírová miska 1070 ml s papírovým víčkem</t>
+          <t>Papírové desky na účet</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>2, 3, 4, 5</t>
+          <t>49</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -1194,7 +1210,7 @@
         </is>
       </c>
       <c r="G19" s="4" t="n">
-        <v>8100</v>
+        <v>500</v>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
@@ -1202,10 +1218,10 @@
         </is>
       </c>
       <c r="I19" s="6" t="n">
-        <v>172</v>
+        <v>22</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>1840</v>
+        <v>100</v>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
@@ -1227,22 +1243,22 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>4823 70 90</t>
+          <t>4823 70 90 00</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Take away box 2oz</t>
+          <t>Take away box 2oz; Coaster</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Jednorázový kelímek 2 oz z bagasy</t>
+          <t>Kelímek 2 oz z bagasy (lisovaná papírovina); Papírový tácek pod sklenici s logem EG</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1, 65</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -1251,7 +1267,7 @@
         </is>
       </c>
       <c r="G20" s="4" t="n">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
@@ -1259,10 +1275,10 @@
         </is>
       </c>
       <c r="I20" s="6" t="n">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>80</v>
+        <v>130</v>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
@@ -1274,7 +1290,11 @@
           <t>Ne</t>
         </is>
       </c>
-      <c r="M20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>Kód dle minulého proclení GAUCHO.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1284,22 +1304,22 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>4823 90 85</t>
+          <t>4823 90 85 80</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Coaster</t>
+          <t>Paper Flags all kinds</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Papírový tácek pod sklenici</t>
+          <t>Papírové vlaječky</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>34</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1308,7 +1328,7 @@
         </is>
       </c>
       <c r="G21" s="4" t="n">
-        <v>500</v>
+        <v>63000</v>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
@@ -1316,10 +1336,10 @@
         </is>
       </c>
       <c r="I21" s="6" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>50</v>
+        <v>1260</v>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
@@ -1331,7 +1351,11 @@
           <t>Ne</t>
         </is>
       </c>
-      <c r="M21" s="4" t="inlineStr"/>
+      <c r="M21" s="4" t="inlineStr">
+        <is>
+          <t>Kód dle minulého proclení GAUCHO.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1341,31 +1365,31 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>4911 99 00</t>
+          <t>6105 10 00</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Paper Flags all kinds</t>
+          <t>Polo; Polo Long Sleeve</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Papírové vlaječky různé</t>
+          <t>Polokošile; Polokošile s dlouhým rukávem</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>67, 69</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>Fabric</t>
         </is>
       </c>
       <c r="G22" s="4" t="n">
-        <v>63000</v>
+        <v>543</v>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
@@ -1373,10 +1397,10 @@
         </is>
       </c>
       <c r="I22" s="6" t="n">
-        <v>24</v>
+        <v>182</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>1260</v>
+        <v>4445</v>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
@@ -1398,22 +1422,22 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>6105 10 00</t>
+          <t>6109 10 00</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Polo; Polo Long Sleeve</t>
+          <t>T-Shirt</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Polokošile; Polokošile s dlouhým rukávem</t>
+          <t>Tričko</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>67, 69</t>
+          <t>68</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1422,7 +1446,7 @@
         </is>
       </c>
       <c r="G23" s="4" t="n">
-        <v>543</v>
+        <v>245</v>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
@@ -1430,10 +1454,10 @@
         </is>
       </c>
       <c r="I23" s="6" t="n">
-        <v>182</v>
+        <v>48</v>
       </c>
       <c r="J23" s="6" t="n">
-        <v>4445</v>
+        <v>1715</v>
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
@@ -1455,22 +1479,22 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>6109 10 00</t>
+          <t>6203 42 35</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>T-Shirt</t>
+          <t>Trouser</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Tričko</t>
+          <t>Kalhoty dlouhé</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>70</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -1479,7 +1503,7 @@
         </is>
       </c>
       <c r="G24" s="4" t="n">
-        <v>245</v>
+        <v>63</v>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
@@ -1487,10 +1511,10 @@
         </is>
       </c>
       <c r="I24" s="6" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="J24" s="6" t="n">
-        <v>1715</v>
+        <v>945</v>
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
@@ -1512,22 +1536,22 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>6203 42 35</t>
+          <t>6205 20 00</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Trouser</t>
+          <t>Floor Uniform - Men</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Kalhoty dlouhé</t>
+          <t>Pánská košile – uniforma obsluhy</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>71</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1536,7 +1560,7 @@
         </is>
       </c>
       <c r="G25" s="4" t="n">
-        <v>63</v>
+        <v>411</v>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
@@ -1544,10 +1568,10 @@
         </is>
       </c>
       <c r="I25" s="6" t="n">
-        <v>30</v>
+        <v>143</v>
       </c>
       <c r="J25" s="6" t="n">
-        <v>945</v>
+        <v>3699</v>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
@@ -1569,22 +1593,22 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>6205 20 00</t>
+          <t>6206 30 00</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Floor Uniform - Men</t>
+          <t>Floor Uniform - Women</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Pánská košile – uniforma obsluhy</t>
+          <t>Dámská košile – uniforma obsluhy</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>72</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1593,7 +1617,7 @@
         </is>
       </c>
       <c r="G26" s="4" t="n">
-        <v>411</v>
+        <v>337</v>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
@@ -1601,10 +1625,10 @@
         </is>
       </c>
       <c r="I26" s="6" t="n">
-        <v>143</v>
+        <v>84</v>
       </c>
       <c r="J26" s="6" t="n">
-        <v>3699</v>
+        <v>3033</v>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
@@ -1626,22 +1650,22 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>6206 30 00</t>
+          <t>6211 32 10</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Floor Uniform - Women</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Dámská košile – uniforma obsluhy</t>
+          <t>Kuchařský rondon</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>66</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -1650,7 +1674,7 @@
         </is>
       </c>
       <c r="G27" s="4" t="n">
-        <v>337</v>
+        <v>317</v>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
@@ -1658,10 +1682,10 @@
         </is>
       </c>
       <c r="I27" s="6" t="n">
-        <v>84</v>
+        <v>144</v>
       </c>
       <c r="J27" s="6" t="n">
-        <v>3033</v>
+        <v>7291</v>
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
@@ -1683,22 +1707,22 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>6211 32 10</t>
+          <t>6211 43 10</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Apron</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Kuchařský rondon</t>
+          <t>Zástěra</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>59</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -1707,7 +1731,7 @@
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>317</v>
+        <v>154</v>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
@@ -1715,10 +1739,10 @@
         </is>
       </c>
       <c r="I28" s="6" t="n">
-        <v>144</v>
+        <v>24</v>
       </c>
       <c r="J28" s="6" t="n">
-        <v>7291</v>
+        <v>1386</v>
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
@@ -1740,22 +1764,22 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>6211 43 10</t>
+          <t>6215 20 00</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Apron</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Zástěra</t>
+          <t>Kravata</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>53</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -1764,7 +1788,7 @@
         </is>
       </c>
       <c r="G29" s="4" t="n">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
@@ -1772,10 +1796,10 @@
         </is>
       </c>
       <c r="I29" s="6" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="J29" s="6" t="n">
-        <v>1386</v>
+        <v>450</v>
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
@@ -1787,7 +1811,11 @@
           <t>Ne</t>
         </is>
       </c>
-      <c r="M29" s="4" t="inlineStr"/>
+      <c r="M29" s="4" t="inlineStr">
+        <is>
+          <t>Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1797,22 +1825,22 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>6215 20 00</t>
+          <t>6216 00 00</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Hot Plate Glove</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Kravata</t>
+          <t>Chňapka / rukavice na horké talíře (pár)</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>60</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -1821,7 +1849,7 @@
         </is>
       </c>
       <c r="G30" s="4" t="n">
-        <v>150</v>
+        <v>30</v>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
@@ -1829,10 +1857,10 @@
         </is>
       </c>
       <c r="I30" s="6" t="n">
-        <v>6</v>
+        <v>2.15</v>
       </c>
       <c r="J30" s="6" t="n">
-        <v>450</v>
+        <v>39</v>
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
@@ -1858,22 +1886,22 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>6216 00 00</t>
+          <t>6302 51 00 90</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Hot Plate Glove</t>
+          <t>Napkin fabric set up</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Chňapka / rukavice na horké talíře (pár)</t>
+          <t>Stolní ubrousky, bavlněná tkanina</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>33</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -1882,7 +1910,7 @@
         </is>
       </c>
       <c r="G31" s="4" t="n">
-        <v>30</v>
+        <v>2000</v>
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
@@ -1890,10 +1918,10 @@
         </is>
       </c>
       <c r="I31" s="6" t="n">
-        <v>2.15</v>
+        <v>122</v>
       </c>
       <c r="J31" s="6" t="n">
-        <v>39</v>
+        <v>7200</v>
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
@@ -1907,7 +1935,7 @@
       </c>
       <c r="M31" s="4" t="inlineStr">
         <is>
-          <t>Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+          <t>Kód dle minulého proclení GAUCHO.</t>
         </is>
       </c>
     </row>
@@ -1919,22 +1947,22 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>6302 51 00</t>
+          <t>6302 60 00</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Napkin fabric set up</t>
+          <t>Black Towel</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Látkový ubrousek</t>
+          <t>Černý ručník</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>62</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -1943,7 +1971,7 @@
         </is>
       </c>
       <c r="G32" s="4" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
@@ -1951,10 +1979,10 @@
         </is>
       </c>
       <c r="I32" s="6" t="n">
-        <v>122</v>
+        <v>37</v>
       </c>
       <c r="J32" s="6" t="n">
-        <v>7200</v>
+        <v>500</v>
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
@@ -1976,22 +2004,22 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>6302 60 00</t>
+          <t>6505 00 30</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Black Towel</t>
+          <t>Cap</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Černý ručník</t>
+          <t>Kšiltovka</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>61</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -2000,7 +2028,7 @@
         </is>
       </c>
       <c r="G33" s="4" t="n">
-        <v>500</v>
+        <v>50</v>
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
@@ -2008,10 +2036,10 @@
         </is>
       </c>
       <c r="I33" s="6" t="n">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="J33" s="6" t="n">
-        <v>500</v>
+        <v>150</v>
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
@@ -2023,7 +2051,11 @@
           <t>Ne</t>
         </is>
       </c>
-      <c r="M33" s="4" t="inlineStr"/>
+      <c r="M33" s="4" t="inlineStr">
+        <is>
+          <t>Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2033,31 +2065,31 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>6505 00 30</t>
+          <t>6912 00 25 10</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Cap</t>
+          <t>FF-bowl big; Side dish bowl &amp; cover; Sauce bowl; Medium plate; Milk jug; Sugar jug  small one; Dressing  jug small one</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Kšiltovka</t>
+          <t>Velká miska salátová, keramika; Přílohová mistička s pokličkou, keramika; Miska na omáčku, keramika; Keramický talíř střední; Malá konvička na mléko, keramika; Malá dóza na cukr, keramika; Malá dóza na omáčky, keramika</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>17, 18, 19, 25, 27, 28, 29</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Fabric</t>
+          <t>Ceramic</t>
         </is>
       </c>
       <c r="G34" s="4" t="n">
-        <v>50</v>
+        <v>670</v>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
@@ -2065,24 +2097,24 @@
         </is>
       </c>
       <c r="I34" s="6" t="n">
-        <v>2</v>
+        <v>250.96</v>
       </c>
       <c r="J34" s="6" t="n">
-        <v>150</v>
+        <v>1684</v>
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="L34" s="4" t="inlineStr">
-        <is>
-          <t>Ne</t>
+      <c r="L34" s="7" t="inlineStr">
+        <is>
+          <t>AD clo na keramické nádobí platí jen při původu ČLR – ověřit, že původ je VN.</t>
         </is>
       </c>
       <c r="M34" s="4" t="inlineStr">
         <is>
-          <t>Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+          <t>Kód dle minulého proclení GAUCHO. Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
         </is>
       </c>
     </row>
@@ -2094,31 +2126,31 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>6911 10 00</t>
+          <t>7010 90 43</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>FF-bowl big; Side dish bowl &amp; cover; Sauce bowl; Medium plate; Milk jug; Sugar jug  small one; Dressing  jug small one</t>
+          <t>Vodka bottle</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Velká keramická mísa; Keramická miska na přílohy s víčkem; Keramická miska na omáčku; Keramický talíř střední; Keramická konvička na mléko; Keramická cukřenka malá; Keramická konvička na dresink malá</t>
+          <t>Skleněná láhev na vodku (prázdná)</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>17, 18, 19, 25, 27, 28, 29</t>
+          <t>16</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Ceramic</t>
+          <t>Glass</t>
         </is>
       </c>
       <c r="G35" s="4" t="n">
-        <v>670</v>
+        <v>1368</v>
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
@@ -2126,26 +2158,22 @@
         </is>
       </c>
       <c r="I35" s="6" t="n">
-        <v>250.96</v>
+        <v>860.5</v>
       </c>
       <c r="J35" s="6" t="n">
-        <v>1684</v>
+        <v>2736</v>
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="L35" s="7" t="inlineStr">
-        <is>
-          <t>AD clo na keramické nádobí platí jen při původu ČLR – ověřit, že původ je VN.</t>
-        </is>
-      </c>
-      <c r="M35" s="4" t="inlineStr">
-        <is>
-          <t>Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
-        </is>
-      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Ne</t>
+        </is>
+      </c>
+      <c r="M35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2155,31 +2183,31 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>7010 90 43</t>
+          <t>7117 19 00</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Vodka bottle</t>
+          <t>Clip</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Skleněná láhev na vodku (prázdná)</t>
+          <t>Kovová spona na kravatu</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>52</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Glass</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="G36" s="4" t="n">
-        <v>1368</v>
+        <v>100</v>
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
@@ -2187,10 +2215,10 @@
         </is>
       </c>
       <c r="I36" s="6" t="n">
-        <v>860.5</v>
+        <v>1.37</v>
       </c>
       <c r="J36" s="6" t="n">
-        <v>2736</v>
+        <v>260</v>
       </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
@@ -2202,7 +2230,11 @@
           <t>Ne</t>
         </is>
       </c>
-      <c r="M36" s="4" t="inlineStr"/>
+      <c r="M36" s="4" t="inlineStr">
+        <is>
+          <t>Ocel/kov: chybí hutní atest (melt &amp; pour). Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2212,27 +2244,27 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>7117 19 00</t>
+          <t>7323 93 00 90</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Clip</t>
+          <t>Paricha; Paricha plate Small; Paricha plate big</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Kovová spona na kravatu</t>
+          <t>Nerezová pánev na uhlíky na udržení teplého masa (parrilla); Nerezový talíř na parrillu malý; Nerezový talíř na parrillu velký</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>36, 37, 38</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Stainless steel</t>
         </is>
       </c>
       <c r="G37" s="4" t="n">
@@ -2244,10 +2276,10 @@
         </is>
       </c>
       <c r="I37" s="6" t="n">
-        <v>1.37</v>
+        <v>38</v>
       </c>
       <c r="J37" s="6" t="n">
-        <v>260</v>
+        <v>440</v>
       </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
@@ -2261,7 +2293,7 @@
       </c>
       <c r="M37" s="4" t="inlineStr">
         <is>
-          <t>Ocel/kov: chybí hutní atest (melt &amp; pour). Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+          <t>Kód dle minulého proclení GAUCHO. Ocel/kov: chybí hutní atest (melt &amp; pour). Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
         </is>
       </c>
     </row>
@@ -2273,31 +2305,31 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>7323 93 10</t>
+          <t>7323 99 00</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Paricha; Paricha plate Small; Paricha plate big</t>
+          <t>Astray</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Nerezový servírovací tác s držadlem (parrilla); Nerezový talíř na parrillu malý; Nerezový talíř na parrillu velký</t>
+          <t>Kovový popelník</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>36, 37, 38</t>
+          <t>31</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Stainless steel</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="G38" s="4" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
@@ -2305,10 +2337,10 @@
         </is>
       </c>
       <c r="I38" s="6" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="J38" s="6" t="n">
-        <v>440</v>
+        <v>4680</v>
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
@@ -2322,7 +2354,7 @@
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>Ocel/kov: chybí hutní atest (melt &amp; pour). Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+          <t>Ocel/kov: chybí hutní atest (melt &amp; pour).</t>
         </is>
       </c>
     </row>
@@ -2334,31 +2366,31 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>7323 99 00</t>
+          <t>8211 91 00</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Astray</t>
+          <t>Steak knives; Setup Knife</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Kovový popelník</t>
+          <t>Nerezový steakový nůž; Nerezový jídelní nůž</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>24, 47</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Stainless steel</t>
         </is>
       </c>
       <c r="G39" s="4" t="n">
-        <v>120</v>
+        <v>1200</v>
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
@@ -2366,10 +2398,10 @@
         </is>
       </c>
       <c r="I39" s="6" t="n">
-        <v>35</v>
+        <v>108.82</v>
       </c>
       <c r="J39" s="6" t="n">
-        <v>4680</v>
+        <v>5660</v>
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
@@ -2383,7 +2415,7 @@
       </c>
       <c r="M39" s="4" t="inlineStr">
         <is>
-          <t>Ocel/kov: chybí hutní atest (melt &amp; pour).</t>
+          <t>Ocel/kov: chybí hutní atest (melt &amp; pour). Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
         </is>
       </c>
     </row>
@@ -2395,22 +2427,22 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>8211 91 00</t>
+          <t>8215 99 10 00</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Steak knives; Setup Knife</t>
+          <t>Salsa spoon espresso; Capucino spoon sauce; Setup folk; Latte spoon; Dessert Spoon; Dessert Fork; Small spoon</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Nerezový steakový nůž; Nerezový jídelní nůž</t>
+          <t>Lžička na espresso, nerez; Lžička na cappuccino, nerez; Vidlička, nerez; Lžička na latte, nerez; Dezertní lžička, nerez; Dezertní vidlička, nerez; Malá lžička, nerez</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>24, 47</t>
+          <t>21, 22, 23, 55, 56, 57, 58</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
@@ -2419,7 +2451,7 @@
         </is>
       </c>
       <c r="G40" s="4" t="n">
-        <v>1200</v>
+        <v>1320</v>
       </c>
       <c r="H40" s="5" t="inlineStr">
         <is>
@@ -2427,10 +2459,10 @@
         </is>
       </c>
       <c r="I40" s="6" t="n">
-        <v>108.82</v>
+        <v>37.03</v>
       </c>
       <c r="J40" s="6" t="n">
-        <v>5660</v>
+        <v>672</v>
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
@@ -2444,7 +2476,7 @@
       </c>
       <c r="M40" s="4" t="inlineStr">
         <is>
-          <t>Ocel/kov: chybí hutní atest (melt &amp; pour). Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+          <t>Kód dle minulého proclení GAUCHO. Ocel/kov: chybí hutní atest (melt &amp; pour). Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
         </is>
       </c>
     </row>
@@ -2456,31 +2488,31 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>8215 99 10</t>
+          <t>8310 00 00</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Salsa spoon espresso; Capucino spoon sauce; Setup folk; Latte spoon; Dessert Spoon; Dessert Fork; Small spoon</t>
+          <t>Round sign; Butcher sign</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Nerezová lžička na espresso / salsu; Nerezová lžička na cappuccino / omáčku; Nerezová jídelní vidlička; Nerezová lžička na latte; Nerezová dezertní lžička; Nerezová dezertní vidlička; Nerezová malá lžička</t>
+          <t>Kulatá reklamní cedule (kov, plast, nerez); Cedule 'Butcher' (kov, plast, nerez)</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>21, 22, 23, 55, 56, 57, 58</t>
+          <t>50, 54</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Stainless steel</t>
+          <t>Metal, plastic and stainless steel</t>
         </is>
       </c>
       <c r="G41" s="4" t="n">
-        <v>1320</v>
+        <v>7</v>
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
@@ -2488,10 +2520,10 @@
         </is>
       </c>
       <c r="I41" s="6" t="n">
-        <v>37.03</v>
+        <v>126</v>
       </c>
       <c r="J41" s="6" t="n">
-        <v>672</v>
+        <v>2140</v>
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
@@ -2505,7 +2537,7 @@
       </c>
       <c r="M41" s="4" t="inlineStr">
         <is>
-          <t>Ocel/kov: chybí hutní atest (melt &amp; pour). Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+          <t>Ocel/kov: chybí hutní atest (melt &amp; pour).</t>
         </is>
       </c>
     </row>
@@ -2517,31 +2549,31 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>8310 00 00</t>
+          <t>8438 10 10</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Round sign; Butcher sign</t>
+          <t>Proofer</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Kulatá reklamní cedule (kov, plast, nerez); Cedule 'Butcher' (kov, plast, nerez)</t>
+          <t>Kynárna na těsto</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>50, 54</t>
+          <t>73</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Metal, plastic and stainless steel</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="G42" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
@@ -2549,10 +2581,10 @@
         </is>
       </c>
       <c r="I42" s="6" t="n">
-        <v>126</v>
+        <v>446</v>
       </c>
       <c r="J42" s="6" t="n">
-        <v>2140</v>
+        <v>1112</v>
       </c>
       <c r="K42" s="4" t="inlineStr">
         <is>
@@ -2578,31 +2610,31 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>8438 10 10</t>
+          <t>9401 61 00 00</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Proofer</t>
+          <t>Low chair</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Kynárna na těsto</t>
+          <t>Nízká židle do restaurace, mořený buk, čalouněná černou koženkou</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>44</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Wood</t>
         </is>
       </c>
       <c r="G43" s="4" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
@@ -2610,10 +2642,10 @@
         </is>
       </c>
       <c r="I43" s="6" t="n">
-        <v>446</v>
+        <v>270</v>
       </c>
       <c r="J43" s="6" t="n">
-        <v>1112</v>
+        <v>2400</v>
       </c>
       <c r="K43" s="4" t="inlineStr">
         <is>
@@ -2627,7 +2659,7 @@
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>Ocel/kov: chybí hutní atest (melt &amp; pour).</t>
+          <t>Kód dle minulého proclení GAUCHO.</t>
         </is>
       </c>
     </row>
@@ -2639,22 +2671,22 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>9401 69 00</t>
+          <t>9403 91 00 90</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Low chair</t>
+          <t>Table face</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Nízká dřevěná židle</t>
+          <t>Stolová deska, dub mořený</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>46</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
@@ -2663,7 +2695,7 @@
         </is>
       </c>
       <c r="G44" s="4" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="H44" s="5" t="inlineStr">
         <is>
@@ -2671,10 +2703,10 @@
         </is>
       </c>
       <c r="I44" s="6" t="n">
-        <v>270</v>
+        <v>432</v>
       </c>
       <c r="J44" s="6" t="n">
-        <v>2400</v>
+        <v>2808</v>
       </c>
       <c r="K44" s="4" t="inlineStr">
         <is>
@@ -2686,7 +2718,11 @@
           <t>Ne</t>
         </is>
       </c>
-      <c r="M44" s="4" t="inlineStr"/>
+      <c r="M44" s="4" t="inlineStr">
+        <is>
+          <t>Kód dle minulého proclení GAUCHO. Ocel/kov: chybí hutní atest (melt &amp; pour).</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -2696,27 +2732,27 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>9403 91 00</t>
+          <t>9403 99 10 90</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Table face</t>
+          <t>Low table leg</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Dřevěná stolní deska</t>
+          <t>Kovová noha od stolu nízká</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>45</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Wood</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="G45" s="4" t="n">
@@ -2728,10 +2764,10 @@
         </is>
       </c>
       <c r="I45" s="6" t="n">
-        <v>432</v>
+        <v>600</v>
       </c>
       <c r="J45" s="6" t="n">
-        <v>2808</v>
+        <v>888</v>
       </c>
       <c r="K45" s="4" t="inlineStr">
         <is>
@@ -2745,7 +2781,7 @@
       </c>
       <c r="M45" s="4" t="inlineStr">
         <is>
-          <t>Ocel/kov: chybí hutní atest (melt &amp; pour).</t>
+          <t>Kód dle minulého proclení GAUCHO. Ocel/kov: chybí hutní atest (melt &amp; pour).</t>
         </is>
       </c>
     </row>
@@ -2757,31 +2793,31 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>9403 99 10</t>
+          <t>9405 21 40 00</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Low table leg</t>
+          <t>Table lamp</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Kovová podnož nízkého stolu</t>
+          <t>Stolní lampička, LED, USB nabíjení</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>35</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Plastic</t>
         </is>
       </c>
       <c r="G46" s="4" t="n">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
@@ -2789,11 +2825,11 @@
         </is>
       </c>
       <c r="I46" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="J46" s="6" t="n">
         <v>600</v>
       </c>
-      <c r="J46" s="6" t="n">
-        <v>888</v>
-      </c>
       <c r="K46" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
@@ -2806,95 +2842,38 @@
       </c>
       <c r="M46" s="4" t="inlineStr">
         <is>
-          <t>Ocel/kov: chybí hutní atest (melt &amp; pour).</t>
+          <t>Kód dle minulého proclení GAUCHO.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>GAUCHO COMPANY LIMITED (HCMC, VN)</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>9405 21 40</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>Table lamp</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>Stolní LED lampa (plast)</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>Plastic</t>
-        </is>
-      </c>
-      <c r="G47" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="H47" s="5" t="inlineStr">
-        <is>
-          <t>CHYBÍ</t>
-        </is>
-      </c>
-      <c r="I47" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="J47" s="6" t="n">
-        <v>600</v>
-      </c>
-      <c r="K47" s="4" t="inlineStr">
-        <is>
-          <t>Ne</t>
-        </is>
-      </c>
-      <c r="L47" s="4" t="inlineStr">
-        <is>
-          <t>Ne</t>
-        </is>
-      </c>
-      <c r="M47" s="4" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="B48" s="9" t="n"/>
-      <c r="C48" s="9" t="n"/>
-      <c r="D48" s="9" t="n"/>
-      <c r="E48" s="9" t="n"/>
-      <c r="F48" s="9" t="n"/>
-      <c r="G48" s="9" t="n"/>
-      <c r="H48" s="10" t="inlineStr">
-        <is>
-          <t>CHYBÍ</t>
-        </is>
-      </c>
-      <c r="I48" s="11">
-        <f>SUM(I10:I47)</f>
+      <c r="B47" s="9" t="n"/>
+      <c r="C47" s="9" t="n"/>
+      <c r="D47" s="9" t="n"/>
+      <c r="E47" s="9" t="n"/>
+      <c r="F47" s="9" t="n"/>
+      <c r="G47" s="9" t="n"/>
+      <c r="H47" s="10" t="inlineStr">
+        <is>
+          <t>CHYBÍ</t>
+        </is>
+      </c>
+      <c r="I47" s="11">
+        <f>SUM(I10:I46)</f>
         <v/>
       </c>
-      <c r="J48" s="11">
-        <f>SUM(J10:J47)</f>
+      <c r="J47" s="11">
+        <f>SUM(J10:J46)</f>
         <v/>
       </c>
-      <c r="K48" s="9" t="n"/>
-      <c r="L48" s="9" t="n"/>
-      <c r="M48" s="9" t="n"/>
+      <c r="K47" s="9" t="n"/>
+      <c r="L47" s="9" t="n"/>
+      <c r="M47" s="9" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
GAUCHO05: keep sender's 6105 10 00 for men's uniform shirt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013kgPsLTRumkJ7okPbw8b4c
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_EL_GAUCHO_CZ_GAUCHO05.xlsx
+++ b/output/HS_Code_Summary_EL_GAUCHO_CZ_GAUCHO05.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M47"/>
+  <dimension ref="A1:M46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1370,17 +1370,17 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Polo; Polo Long Sleeve</t>
+          <t>Polo; Polo Long Sleeve; Floor Uniform - Men</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Polokošile; Polokošile s dlouhým rukávem</t>
+          <t>Polokošile; Polokošile s dlouhým rukávem; Pánská košile – uniforma obsluhy</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>67, 69</t>
+          <t>67, 69, 71</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1389,7 +1389,7 @@
         </is>
       </c>
       <c r="G22" s="4" t="n">
-        <v>543</v>
+        <v>954</v>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
@@ -1397,10 +1397,10 @@
         </is>
       </c>
       <c r="I22" s="6" t="n">
-        <v>182</v>
+        <v>325</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>4445</v>
+        <v>8144</v>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
@@ -1536,22 +1536,22 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>6205 20 00</t>
+          <t>6206 30 00</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Floor Uniform - Men</t>
+          <t>Floor Uniform - Women</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Pánská košile – uniforma obsluhy</t>
+          <t>Dámská košile – uniforma obsluhy</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>72</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="G25" s="4" t="n">
-        <v>411</v>
+        <v>337</v>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
@@ -1568,10 +1568,10 @@
         </is>
       </c>
       <c r="I25" s="6" t="n">
-        <v>143</v>
+        <v>84</v>
       </c>
       <c r="J25" s="6" t="n">
-        <v>3699</v>
+        <v>3033</v>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
@@ -1593,22 +1593,22 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>6206 30 00</t>
+          <t>6211 32 10</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Floor Uniform - Women</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Dámská košile – uniforma obsluhy</t>
+          <t>Kuchařský rondon</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>66</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1617,7 +1617,7 @@
         </is>
       </c>
       <c r="G26" s="4" t="n">
-        <v>337</v>
+        <v>317</v>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
@@ -1625,10 +1625,10 @@
         </is>
       </c>
       <c r="I26" s="6" t="n">
-        <v>84</v>
+        <v>144</v>
       </c>
       <c r="J26" s="6" t="n">
-        <v>3033</v>
+        <v>7291</v>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>6211 32 10</t>
+          <t>6211 43 10</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Apron</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Kuchařský rondon</t>
+          <t>Zástěra</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>59</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -1674,7 +1674,7 @@
         </is>
       </c>
       <c r="G27" s="4" t="n">
-        <v>317</v>
+        <v>154</v>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
@@ -1682,10 +1682,10 @@
         </is>
       </c>
       <c r="I27" s="6" t="n">
-        <v>144</v>
+        <v>24</v>
       </c>
       <c r="J27" s="6" t="n">
-        <v>7291</v>
+        <v>1386</v>
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
@@ -1707,22 +1707,22 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>6211 43 10</t>
+          <t>6215 20 00</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Apron</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Zástěra</t>
+          <t>Kravata</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>53</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -1731,7 +1731,7 @@
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
@@ -1739,10 +1739,10 @@
         </is>
       </c>
       <c r="I28" s="6" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="J28" s="6" t="n">
-        <v>1386</v>
+        <v>450</v>
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
@@ -1754,7 +1754,11 @@
           <t>Ne</t>
         </is>
       </c>
-      <c r="M28" s="4" t="inlineStr"/>
+      <c r="M28" s="4" t="inlineStr">
+        <is>
+          <t>Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1764,22 +1768,22 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>6215 20 00</t>
+          <t>6216 00 00</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Hot Plate Glove</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Kravata</t>
+          <t>Chňapka / rukavice na horké talíře (pár)</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>60</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -1788,7 +1792,7 @@
         </is>
       </c>
       <c r="G29" s="4" t="n">
-        <v>150</v>
+        <v>30</v>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
@@ -1796,10 +1800,10 @@
         </is>
       </c>
       <c r="I29" s="6" t="n">
-        <v>6</v>
+        <v>2.15</v>
       </c>
       <c r="J29" s="6" t="n">
-        <v>450</v>
+        <v>39</v>
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
@@ -1825,22 +1829,22 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>6216 00 00</t>
+          <t>6302 51 00 90</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Hot Plate Glove</t>
+          <t>Napkin fabric set up</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Chňapka / rukavice na horké talíře (pár)</t>
+          <t>Stolní ubrousky, bavlněná tkanina</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>33</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -1849,7 +1853,7 @@
         </is>
       </c>
       <c r="G30" s="4" t="n">
-        <v>30</v>
+        <v>2000</v>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
@@ -1857,10 +1861,10 @@
         </is>
       </c>
       <c r="I30" s="6" t="n">
-        <v>2.15</v>
+        <v>122</v>
       </c>
       <c r="J30" s="6" t="n">
-        <v>39</v>
+        <v>7200</v>
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
@@ -1874,7 +1878,7 @@
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+          <t>Kód dle minulého proclení GAUCHO.</t>
         </is>
       </c>
     </row>
@@ -1886,22 +1890,22 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>6302 51 00 90</t>
+          <t>6302 60 00</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Napkin fabric set up</t>
+          <t>Black Towel</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Stolní ubrousky, bavlněná tkanina</t>
+          <t>Černý ručník</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>62</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -1910,7 +1914,7 @@
         </is>
       </c>
       <c r="G31" s="4" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
@@ -1918,10 +1922,10 @@
         </is>
       </c>
       <c r="I31" s="6" t="n">
-        <v>122</v>
+        <v>37</v>
       </c>
       <c r="J31" s="6" t="n">
-        <v>7200</v>
+        <v>500</v>
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
@@ -1933,11 +1937,7 @@
           <t>Ne</t>
         </is>
       </c>
-      <c r="M31" s="4" t="inlineStr">
-        <is>
-          <t>Kód dle minulého proclení GAUCHO.</t>
-        </is>
-      </c>
+      <c r="M31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1947,22 +1947,22 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>6302 60 00</t>
+          <t>6505 00 30</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Black Towel</t>
+          <t>Cap</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Černý ručník</t>
+          <t>Kšiltovka</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>61</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="G32" s="4" t="n">
-        <v>500</v>
+        <v>50</v>
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
@@ -1979,10 +1979,10 @@
         </is>
       </c>
       <c r="I32" s="6" t="n">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="J32" s="6" t="n">
-        <v>500</v>
+        <v>150</v>
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
@@ -1994,7 +1994,11 @@
           <t>Ne</t>
         </is>
       </c>
-      <c r="M32" s="4" t="inlineStr"/>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t>Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -2004,31 +2008,31 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>6505 00 30</t>
+          <t>6912 00 25 10</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Cap</t>
+          <t>FF-bowl big; Side dish bowl &amp; cover; Sauce bowl; Medium plate; Milk jug; Sugar jug  small one; Dressing  jug small one</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Kšiltovka</t>
+          <t>Velká miska salátová, keramika; Přílohová mistička s pokličkou, keramika; Miska na omáčku, keramika; Keramický talíř střední; Malá konvička na mléko, keramika; Malá dóza na cukr, keramika; Malá dóza na omáčky, keramika</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>17, 18, 19, 25, 27, 28, 29</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Fabric</t>
+          <t>Ceramic</t>
         </is>
       </c>
       <c r="G33" s="4" t="n">
-        <v>50</v>
+        <v>670</v>
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
@@ -2036,24 +2040,24 @@
         </is>
       </c>
       <c r="I33" s="6" t="n">
-        <v>2</v>
+        <v>250.96</v>
       </c>
       <c r="J33" s="6" t="n">
-        <v>150</v>
+        <v>1684</v>
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="L33" s="4" t="inlineStr">
-        <is>
-          <t>Ne</t>
+      <c r="L33" s="7" t="inlineStr">
+        <is>
+          <t>AD clo na keramické nádobí platí jen při původu ČLR – ověřit, že původ je VN.</t>
         </is>
       </c>
       <c r="M33" s="4" t="inlineStr">
         <is>
-          <t>Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+          <t>Kód dle minulého proclení GAUCHO. Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
         </is>
       </c>
     </row>
@@ -2065,31 +2069,31 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>6912 00 25 10</t>
+          <t>7010 90 43</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>FF-bowl big; Side dish bowl &amp; cover; Sauce bowl; Medium plate; Milk jug; Sugar jug  small one; Dressing  jug small one</t>
+          <t>Vodka bottle</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Velká miska salátová, keramika; Přílohová mistička s pokličkou, keramika; Miska na omáčku, keramika; Keramický talíř střední; Malá konvička na mléko, keramika; Malá dóza na cukr, keramika; Malá dóza na omáčky, keramika</t>
+          <t>Skleněná láhev na vodku (prázdná)</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>17, 18, 19, 25, 27, 28, 29</t>
+          <t>16</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Ceramic</t>
+          <t>Glass</t>
         </is>
       </c>
       <c r="G34" s="4" t="n">
-        <v>670</v>
+        <v>1368</v>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
@@ -2097,26 +2101,22 @@
         </is>
       </c>
       <c r="I34" s="6" t="n">
-        <v>250.96</v>
+        <v>860.5</v>
       </c>
       <c r="J34" s="6" t="n">
-        <v>1684</v>
+        <v>2736</v>
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="L34" s="7" t="inlineStr">
-        <is>
-          <t>AD clo na keramické nádobí platí jen při původu ČLR – ověřit, že původ je VN.</t>
-        </is>
-      </c>
-      <c r="M34" s="4" t="inlineStr">
-        <is>
-          <t>Kód dle minulého proclení GAUCHO. Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
-        </is>
-      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>Ne</t>
+        </is>
+      </c>
+      <c r="M34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2126,31 +2126,31 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>7010 90 43</t>
+          <t>7117 19 00</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Vodka bottle</t>
+          <t>Clip</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Skleněná láhev na vodku (prázdná)</t>
+          <t>Kovová spona na kravatu</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>52</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Glass</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="G35" s="4" t="n">
-        <v>1368</v>
+        <v>100</v>
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
@@ -2158,10 +2158,10 @@
         </is>
       </c>
       <c r="I35" s="6" t="n">
-        <v>860.5</v>
+        <v>1.37</v>
       </c>
       <c r="J35" s="6" t="n">
-        <v>2736</v>
+        <v>260</v>
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
@@ -2173,7 +2173,11 @@
           <t>Ne</t>
         </is>
       </c>
-      <c r="M35" s="4" t="inlineStr"/>
+      <c r="M35" s="4" t="inlineStr">
+        <is>
+          <t>Ocel/kov: chybí hutní atest (melt &amp; pour). Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2183,27 +2187,27 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>7117 19 00</t>
+          <t>7323 93 00 90</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Clip</t>
+          <t>Paricha; Paricha plate Small; Paricha plate big</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Kovová spona na kravatu</t>
+          <t>Nerezová pánev na uhlíky na udržení teplého masa (parrilla); Nerezový talíř na parrillu malý; Nerezový talíř na parrillu velký</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>36, 37, 38</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Stainless steel</t>
         </is>
       </c>
       <c r="G36" s="4" t="n">
@@ -2215,10 +2219,10 @@
         </is>
       </c>
       <c r="I36" s="6" t="n">
-        <v>1.37</v>
+        <v>38</v>
       </c>
       <c r="J36" s="6" t="n">
-        <v>260</v>
+        <v>440</v>
       </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
@@ -2232,7 +2236,7 @@
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>Ocel/kov: chybí hutní atest (melt &amp; pour). Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+          <t>Kód dle minulého proclení GAUCHO. Ocel/kov: chybí hutní atest (melt &amp; pour). Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
         </is>
       </c>
     </row>
@@ -2244,31 +2248,31 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>7323 93 00 90</t>
+          <t>7323 99 00</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Paricha; Paricha plate Small; Paricha plate big</t>
+          <t>Astray</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Nerezová pánev na uhlíky na udržení teplého masa (parrilla); Nerezový talíř na parrillu malý; Nerezový talíř na parrillu velký</t>
+          <t>Kovový popelník</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>36, 37, 38</t>
+          <t>31</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Stainless steel</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="G37" s="4" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
@@ -2276,10 +2280,10 @@
         </is>
       </c>
       <c r="I37" s="6" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="J37" s="6" t="n">
-        <v>440</v>
+        <v>4680</v>
       </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
@@ -2293,7 +2297,7 @@
       </c>
       <c r="M37" s="4" t="inlineStr">
         <is>
-          <t>Kód dle minulého proclení GAUCHO. Ocel/kov: chybí hutní atest (melt &amp; pour). Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+          <t>Ocel/kov: chybí hutní atest (melt &amp; pour).</t>
         </is>
       </c>
     </row>
@@ -2305,31 +2309,31 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>7323 99 00</t>
+          <t>8211 91 00</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Astray</t>
+          <t>Steak knives; Setup Knife</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Kovový popelník</t>
+          <t>Nerezový steakový nůž; Nerezový jídelní nůž</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>24, 47</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Stainless steel</t>
         </is>
       </c>
       <c r="G38" s="4" t="n">
-        <v>120</v>
+        <v>1200</v>
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
@@ -2337,10 +2341,10 @@
         </is>
       </c>
       <c r="I38" s="6" t="n">
-        <v>35</v>
+        <v>108.82</v>
       </c>
       <c r="J38" s="6" t="n">
-        <v>4680</v>
+        <v>5660</v>
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
@@ -2354,7 +2358,7 @@
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>Ocel/kov: chybí hutní atest (melt &amp; pour).</t>
+          <t>Ocel/kov: chybí hutní atest (melt &amp; pour). Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
         </is>
       </c>
     </row>
@@ -2366,22 +2370,22 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>8211 91 00</t>
+          <t>8215 99 10 00</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Steak knives; Setup Knife</t>
+          <t>Salsa spoon espresso; Capucino spoon sauce; Setup folk; Latte spoon; Dessert Spoon; Dessert Fork; Small spoon</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Nerezový steakový nůž; Nerezový jídelní nůž</t>
+          <t>Lžička na espresso, nerez; Lžička na cappuccino, nerez; Vidlička, nerez; Lžička na latte, nerez; Dezertní lžička, nerez; Dezertní vidlička, nerez; Malá lžička, nerez</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>24, 47</t>
+          <t>21, 22, 23, 55, 56, 57, 58</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
@@ -2390,7 +2394,7 @@
         </is>
       </c>
       <c r="G39" s="4" t="n">
-        <v>1200</v>
+        <v>1320</v>
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
@@ -2398,10 +2402,10 @@
         </is>
       </c>
       <c r="I39" s="6" t="n">
-        <v>108.82</v>
+        <v>37.03</v>
       </c>
       <c r="J39" s="6" t="n">
-        <v>5660</v>
+        <v>672</v>
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
@@ -2415,7 +2419,7 @@
       </c>
       <c r="M39" s="4" t="inlineStr">
         <is>
-          <t>Ocel/kov: chybí hutní atest (melt &amp; pour). Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+          <t>Kód dle minulého proclení GAUCHO. Ocel/kov: chybí hutní atest (melt &amp; pour). Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
         </is>
       </c>
     </row>
@@ -2427,31 +2431,31 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>8215 99 10 00</t>
+          <t>8310 00 00</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Salsa spoon espresso; Capucino spoon sauce; Setup folk; Latte spoon; Dessert Spoon; Dessert Fork; Small spoon</t>
+          <t>Round sign; Butcher sign</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Lžička na espresso, nerez; Lžička na cappuccino, nerez; Vidlička, nerez; Lžička na latte, nerez; Dezertní lžička, nerez; Dezertní vidlička, nerez; Malá lžička, nerez</t>
+          <t>Kulatá reklamní cedule (kov, plast, nerez); Cedule 'Butcher' (kov, plast, nerez)</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>21, 22, 23, 55, 56, 57, 58</t>
+          <t>50, 54</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Stainless steel</t>
+          <t>Metal, plastic and stainless steel</t>
         </is>
       </c>
       <c r="G40" s="4" t="n">
-        <v>1320</v>
+        <v>7</v>
       </c>
       <c r="H40" s="5" t="inlineStr">
         <is>
@@ -2459,10 +2463,10 @@
         </is>
       </c>
       <c r="I40" s="6" t="n">
-        <v>37.03</v>
+        <v>126</v>
       </c>
       <c r="J40" s="6" t="n">
-        <v>672</v>
+        <v>2140</v>
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
@@ -2476,7 +2480,7 @@
       </c>
       <c r="M40" s="4" t="inlineStr">
         <is>
-          <t>Kód dle minulého proclení GAUCHO. Ocel/kov: chybí hutní atest (melt &amp; pour). Hrubá hmotnost částečně rozpočtena podle hodnoty (sdílený karton).</t>
+          <t>Ocel/kov: chybí hutní atest (melt &amp; pour).</t>
         </is>
       </c>
     </row>
@@ -2488,31 +2492,31 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>8310 00 00</t>
+          <t>8438 10 10</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Round sign; Butcher sign</t>
+          <t>Proofer</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Kulatá reklamní cedule (kov, plast, nerez); Cedule 'Butcher' (kov, plast, nerez)</t>
+          <t>Kynárna na těsto</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>50, 54</t>
+          <t>73</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Metal, plastic and stainless steel</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="G41" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
@@ -2520,10 +2524,10 @@
         </is>
       </c>
       <c r="I41" s="6" t="n">
-        <v>126</v>
+        <v>446</v>
       </c>
       <c r="J41" s="6" t="n">
-        <v>2140</v>
+        <v>1112</v>
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
@@ -2549,31 +2553,31 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>8438 10 10</t>
+          <t>9401 61 00 00</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Proofer</t>
+          <t>Low chair</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Kynárna na těsto</t>
+          <t>Nízká židle do restaurace, mořený buk, čalouněná černou koženkou</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>44</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Wood</t>
         </is>
       </c>
       <c r="G42" s="4" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
@@ -2581,10 +2585,10 @@
         </is>
       </c>
       <c r="I42" s="6" t="n">
-        <v>446</v>
+        <v>270</v>
       </c>
       <c r="J42" s="6" t="n">
-        <v>1112</v>
+        <v>2400</v>
       </c>
       <c r="K42" s="4" t="inlineStr">
         <is>
@@ -2598,7 +2602,7 @@
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>Ocel/kov: chybí hutní atest (melt &amp; pour).</t>
+          <t>Kód dle minulého proclení GAUCHO.</t>
         </is>
       </c>
     </row>
@@ -2610,22 +2614,22 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>9401 61 00 00</t>
+          <t>9403 91 00 90</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Low chair</t>
+          <t>Table face</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Nízká židle do restaurace, mořený buk, čalouněná černou koženkou</t>
+          <t>Stolová deska, dub mořený</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>46</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
@@ -2634,7 +2638,7 @@
         </is>
       </c>
       <c r="G43" s="4" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
@@ -2642,10 +2646,10 @@
         </is>
       </c>
       <c r="I43" s="6" t="n">
-        <v>270</v>
+        <v>432</v>
       </c>
       <c r="J43" s="6" t="n">
-        <v>2400</v>
+        <v>2808</v>
       </c>
       <c r="K43" s="4" t="inlineStr">
         <is>
@@ -2659,7 +2663,7 @@
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>Kód dle minulého proclení GAUCHO.</t>
+          <t>Kód dle minulého proclení GAUCHO. Ocel/kov: chybí hutní atest (melt &amp; pour).</t>
         </is>
       </c>
     </row>
@@ -2671,27 +2675,27 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>9403 91 00 90</t>
+          <t>9403 99 10 90</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Table face</t>
+          <t>Low table leg</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Stolová deska, dub mořený</t>
+          <t>Kovová noha od stolu nízká</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>45</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Wood</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="G44" s="4" t="n">
@@ -2703,10 +2707,10 @@
         </is>
       </c>
       <c r="I44" s="6" t="n">
-        <v>432</v>
+        <v>600</v>
       </c>
       <c r="J44" s="6" t="n">
-        <v>2808</v>
+        <v>888</v>
       </c>
       <c r="K44" s="4" t="inlineStr">
         <is>
@@ -2732,31 +2736,31 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>9403 99 10 90</t>
+          <t>9405 21 40 00</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Low table leg</t>
+          <t>Table lamp</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Kovová noha od stolu nízká</t>
+          <t>Stolní lampička, LED, USB nabíjení</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>35</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Plastic</t>
         </is>
       </c>
       <c r="G45" s="4" t="n">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
@@ -2764,11 +2768,11 @@
         </is>
       </c>
       <c r="I45" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="J45" s="6" t="n">
         <v>600</v>
       </c>
-      <c r="J45" s="6" t="n">
-        <v>888</v>
-      </c>
       <c r="K45" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
@@ -2781,99 +2785,38 @@
       </c>
       <c r="M45" s="4" t="inlineStr">
         <is>
-          <t>Kód dle minulého proclení GAUCHO. Ocel/kov: chybí hutní atest (melt &amp; pour).</t>
+          <t>Kód dle minulého proclení GAUCHO.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>GAUCHO COMPANY LIMITED (HCMC, VN)</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>9405 21 40 00</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>Table lamp</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>Stolní lampička, LED, USB nabíjení</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>Plastic</t>
-        </is>
-      </c>
-      <c r="G46" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="H46" s="5" t="inlineStr">
-        <is>
-          <t>CHYBÍ</t>
-        </is>
-      </c>
-      <c r="I46" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="J46" s="6" t="n">
-        <v>600</v>
-      </c>
-      <c r="K46" s="4" t="inlineStr">
-        <is>
-          <t>Ne</t>
-        </is>
-      </c>
-      <c r="L46" s="4" t="inlineStr">
-        <is>
-          <t>Ne</t>
-        </is>
-      </c>
-      <c r="M46" s="4" t="inlineStr">
-        <is>
-          <t>Kód dle minulého proclení GAUCHO.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="B47" s="9" t="n"/>
-      <c r="C47" s="9" t="n"/>
-      <c r="D47" s="9" t="n"/>
-      <c r="E47" s="9" t="n"/>
-      <c r="F47" s="9" t="n"/>
-      <c r="G47" s="9" t="n"/>
-      <c r="H47" s="10" t="inlineStr">
-        <is>
-          <t>CHYBÍ</t>
-        </is>
-      </c>
-      <c r="I47" s="11">
-        <f>SUM(I10:I46)</f>
+      <c r="B46" s="9" t="n"/>
+      <c r="C46" s="9" t="n"/>
+      <c r="D46" s="9" t="n"/>
+      <c r="E46" s="9" t="n"/>
+      <c r="F46" s="9" t="n"/>
+      <c r="G46" s="9" t="n"/>
+      <c r="H46" s="10" t="inlineStr">
+        <is>
+          <t>CHYBÍ</t>
+        </is>
+      </c>
+      <c r="I46" s="11">
+        <f>SUM(I10:I45)</f>
         <v/>
       </c>
-      <c r="J47" s="11">
-        <f>SUM(J10:J46)</f>
+      <c r="J46" s="11">
+        <f>SUM(J10:J45)</f>
         <v/>
       </c>
-      <c r="K47" s="9" t="n"/>
-      <c r="L47" s="9" t="n"/>
-      <c r="M47" s="9" t="n"/>
+      <c r="K46" s="9" t="n"/>
+      <c r="L46" s="9" t="n"/>
+      <c r="M46" s="9" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>